<commit_message>
Polish QIB/207 reconciliation worksheet formatting
Navy/gold title bars, frozen headers, auto-filter, zebra striping,
red negative amounts, totals rows, tuned column widths, RTL layout.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BtLCoHFw5VydjRz1BFxPhU
</commit_message>
<xml_diff>
--- a/Worksheet_QIB207_Rec.xlsx
+++ b/Worksheet_QIB207_Rec.xlsx
@@ -9,9 +9,12 @@
   <sheets>
     <sheet name="ملخص" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="حركات بنك ناقصة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="قيود دفتر بدون أصل بنكي" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="قيود دفتر بدون أصل" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'حركات بنك ناقصة'!$A$3:$F$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'قيود دفتر بدون أصل'!$A$3:$G$23</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +31,46 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="13"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -46,12 +79,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C0392B"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E7A46"/>
+        <fgColor rgb="00C9A227"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF0FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,32 +108,64 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00AFBCD6"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00AFBCD6"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00AFBCD6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00AFBCD6"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,95 +535,101 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ورقة مطابقة QIB/207 للمحاسب — حركات غير متطابقة</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+          <t>ورقة مطابقة  QIB / 207  —  للمحاسب</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الأساس: كشف حساب QIB/207 الرسمي  •  الرصيد النهائي 428,636.69 (GL=Dashboard=Bank)  •  10/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>رصيد QIB النهائي</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>428,636.69 (GL=Dashboard=Bank) ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>428,636.69  —  GL = Dashboard = Bank  ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>الوضع</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>الرصيد مطابق، لكن بالمقاصّة؛ الحركات أدناه غير متطابقة سطر بسطر</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>حركات بنك بدون مقابل في الدفتر</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>23 حركة   (صافي -94,244.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>قيود دفتر بدون أصل بنكي</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>20 قيد   (صافي -171,239.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>المطلوب من المحاسب</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>تأكيد كل حركة بنك (مسجّلة بصيغة مختلفة أم ناقصة فعلاً)، تسجيل الناقص الحقيقي، ومراجعة قيود الدفتر بدون أصل بنكي</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>الرصيد مطابق لكن بالمقاصّة؛ الحركات التالية غير متطابقة سطر بسطر وتحتاج مطابقة/تصنيف</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>حركات بنك بدون مقابل في الدفتر (يرجّح غير مسجّلة)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>23  | صافي -94,244.79</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>قيود بالدفتر بدون مقابل في البنك (تحتاج مراجعة)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>20  | صافي -171,239.31</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>المطلوب من المحاسب</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>لكل حركة بنك: تأكيد إن كانت مسجّلة بصيغة مختلفة أم لا، وتسجيل الناقص الحقيقي؛ ومراجعة قيود الدفتر بدون أصل بنكي. الأساس = كشف البنك.</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>لا تمسّ القيد الافتتاحي؛ كل قيد يُرفق به كشف البنك + تبرير</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -559,435 +640,543 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>حركات بنك بدون مقابل في الدفتر  (للتصنيف)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الأساس: كشف حساب QIB/207 الرسمي  •  الرصيد النهائي 428,636.69 (GL=Dashboard=Bank)  •  10/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>المرجع</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>المبلغ (دائن-مدين)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>مطابق في الدفتر؟ (للمحاسب)</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>الحساب المقابل الصحيح (للمحاسب)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>مطابق في الدفتر؟</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>الحساب المقابل الصحيح</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>FT26175BL6F3</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D4" s="7" t="n">
         <v>500000</v>
       </c>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>FT261252GMPM</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D5" s="10" t="n">
         <v>-203279.31</v>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>FT26277YH6C1</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D6" s="10" t="n">
         <v>-180551</v>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>FT262783DZ6L</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D7" s="11" t="n">
         <v>160335.52</v>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>FT262780TCYF</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D8" s="10" t="n">
         <v>-100000</v>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>FT2627761P57</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D9" s="10" t="n">
         <v>-71552</v>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>FT26275X0VYT</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D10" s="10" t="n">
         <v>-60000</v>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>FT262751YTBM</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D11" s="10" t="n">
         <v>-25000</v>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>FT26275LTGNY</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D12" s="10" t="n">
         <v>-22500</v>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>FT262778RNG9</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D13" s="10" t="n">
         <v>-22000</v>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>FT26277XG7K9</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D14" s="10" t="n">
         <v>-19835</v>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>FT262777R1LL</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="D15" s="10" t="n">
         <v>-14407</v>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>FT26274G6WKK</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D16" s="10" t="n">
         <v>-11000</v>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>FT26275RTD8M</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="D17" s="10" t="n">
         <v>-9560</v>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>FT26277VGKZY</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="D18" s="10" t="n">
         <v>-7774</v>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>FT26241P37MG</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="D19" s="10" t="n">
         <v>-2000</v>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>FT26241YKZGR</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="D20" s="10" t="n">
         <v>-1000</v>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>FT26256MRG30</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="D21" s="10" t="n">
         <v>-1000</v>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>FT2625299C3G</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="D22" s="10" t="n">
         <v>-950</v>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>FT262569CH26</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="D23" s="10" t="n">
         <v>-836</v>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>FT262568DBX3</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="D24" s="10" t="n">
         <v>-450</v>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>FT2625637D8J</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="D25" s="10" t="n">
         <v>-443</v>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr"/>
+      <c r="F25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>FT262563J6LK</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="D26" s="10" t="n">
         <v>-443</v>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>-94244.78999999999</v>
+      </c>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:F26"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -998,571 +1187,671 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>قيود بالدفتر بدون مقابل في كشف البنك  (للمراجعة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الأساس: كشف حساب QIB/207 الرسمي  •  الرصيد النهائي 428,636.69 (GL=Dashboard=Bank)  •  10/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>التاريخ</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>رقم القيد</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>المصدر</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>المبلغ</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>البيان</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>سليم/يُصحّح؟ (للمحاسب)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>سليم / يُصحّح؟</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00583</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E4" s="10" t="n">
         <v>-30963</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Being Payment from QIB Bank A/c 60207 to Elec</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Being Payment from QIB Bank A/c 60207 to Electrici</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00362</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="E5" s="15" t="n">
         <v>-27232</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Being Payment from QIB Bank A/c 60207 to Elec</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Being Payment from QIB Bank A/c 60207 to Electrici</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00866</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E6" s="10" t="n">
         <v>-24015</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Being Payment from QIB Bank A/c 60207 to Elec</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Being Payment from QIB Bank A/c 60207 to Electrici</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00865</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E7" s="15" t="n">
         <v>-17854</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>BEING ELECTRIC &amp; WIFI PAID FOR THE MONTH OF A</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEING ELECTRIC &amp; WIFI PAID FOR THE MONTH OF APRIL </t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00700</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E8" s="10" t="n">
         <v>-16116</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>general expenses</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>MISC/2026/10/0006</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E9" s="15" t="n">
         <v>-12000</v>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Outward QATCH Transfer AL SARH REAL ES 
-QA58C</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+QA58CBQA00</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00855</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E10" s="10" t="n">
         <v>-12000</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>salary expenses ANAS IBRAHIM</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00876</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E11" s="15" t="n">
         <v>-10981</v>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Outward QATCH Transfer Service Fees and Charg</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Outward QATCH Transfer Service Fees and Charges Pa</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00701</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E12" s="10" t="n">
         <v>-7110</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>general expenses</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00874</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E13" s="15" t="n">
         <v>-5210</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Outward QATCH Transfer Service Fees and Charg</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Outward QATCH Transfer Service Fees and Charges Pa</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00875</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E14" s="10" t="n">
         <v>-3980</v>
       </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Outward QATCH Transfer Service Fees and Charg</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Outward QATCH Transfer Service Fees and Charges Pa</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00002</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>قديم100008</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E15" s="15" t="n">
         <v>-3279.31</v>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Charge Supplier payment</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00859</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E16" s="10" t="n">
         <v>-120</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>QATCH Charges</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00826</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E17" s="15" t="n">
         <v>-100</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>QATCH Charges</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00757</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E18" s="10" t="n">
         <v>-100</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>QATCH Charges</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00837</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E19" s="15" t="n">
         <v>-100</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>QATCH Charges</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/00814</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="E20" s="10" t="n">
         <v>-40</v>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Being Payment from QIB Bank A/c 60207 to Outg</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Being Payment from QIB Bank A/c 60207 to Outgoing </t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/01104</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="E21" s="15" t="n">
         <v>-20</v>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">QATCH Charges    </t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>QIB/2026/01103</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="E22" s="10" t="n">
         <v>-20</v>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">QATCH Charges    </t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>QIB/2026/00383</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>جديد100001</t>
         </is>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="E23" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>QIB CREDITED DATED ON 22 JUNE 2026 BASED ODOO</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>QIB CREDITED DATED ON 22 JUNE 2026 BASED ODOO SALE</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>-171239.31</v>
+      </c>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A3:G23"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>